<commit_message>
fixed templlates for Excel compatibility
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/protocol/PanAm3Medals-A4.xlsx
+++ b/owlcms/src/main/resources/templates/protocol/PanAm3Medals-A4.xlsx
@@ -484,7 +484,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" ns1:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="_-#,##0;[Red]\(#,##0\);\-"/>
     <numFmt numFmtId="165" formatCode="0;\(0\);\-"/>
@@ -2793,7 +2793,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns4="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns4="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns2:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Feuil4">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>

</xml_diff>